<commit_message>
Updated files for compatibility with previous commit
</commit_message>
<xml_diff>
--- a/Algorithm/Acquisition/signalData.xlsx
+++ b/Algorithm/Acquisition/signalData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cranfield-my.sharepoint.com/personal/a_lavinorejas_261_cranfield_ac_uk/Documents/Documents/Group Design Project/Cranfield-LEO-PNT/Algorithm/Acquisition/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{31AC4230-72C4-4582-8E31-DEF67DFFC137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{31AC4230-72C4-4582-8E31-DEF67DFFC137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{524F49DA-ADC2-4C4B-BAB8-B011924C8369}"/>
   <bookViews>
     <workbookView xWindow="2933" yWindow="2933" windowWidth="19200" windowHeight="9980" xr2:uid="{C1A3185A-F3C0-4606-B2D6-D4D09FADDBA2}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>ID</t>
   </si>
@@ -51,6 +51,15 @@
   </si>
   <si>
     <t>rx_stream-320.00-1975.00-2-nvme2.56-10db.bin</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>Oscillator signal, should not have any Doppler</t>
+  </si>
+  <si>
+    <t>Signal captured, expect Doppler</t>
   </si>
 </sst>
 </file>
@@ -431,15 +440,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C04845A8-D2B3-4AA5-B1E2-4210EB6AE0BD}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="39.5859375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.46875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.9375" customWidth="1"/>
+    <col min="4" max="4" width="36.5859375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -449,8 +459,11 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A2">
         <v>0</v>
       </c>
@@ -461,8 +474,11 @@
         <f>500000000</f>
         <v>500000000</v>
       </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A3">
         <v>1</v>
       </c>
@@ -472,6 +488,9 @@
       <c r="C3">
         <f>320000000</f>
         <v>320000000</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new signal to excel
</commit_message>
<xml_diff>
--- a/Algorithm/Acquisition/signalData.xlsx
+++ b/Algorithm/Acquisition/signalData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cranfield-my.sharepoint.com/personal/a_lavinorejas_261_cranfield_ac_uk/Documents/Documents/Group Design Project/Cranfield-LEO-PNT/Algorithm/Acquisition/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{31AC4230-72C4-4582-8E31-DEF67DFFC137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{524F49DA-ADC2-4C4B-BAB8-B011924C8369}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{31AC4230-72C4-4582-8E31-DEF67DFFC137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{472921F9-5837-43F7-A322-0337B65D3855}"/>
   <bookViews>
-    <workbookView xWindow="2933" yWindow="2933" windowWidth="19200" windowHeight="9980" xr2:uid="{C1A3185A-F3C0-4606-B2D6-D4D09FADDBA2}"/>
+    <workbookView xWindow="1100" yWindow="1100" windowWidth="19200" windowHeight="9980" xr2:uid="{C1A3185A-F3C0-4606-B2D6-D4D09FADDBA2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>ID</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>Signal captured, expect Doppler</t>
+  </si>
+  <si>
+    <t>rx_stream-360.00-1975.00-1-10dB-11032026T110930.bin</t>
+  </si>
+  <si>
+    <t>SymbolFreq</t>
   </si>
 </sst>
 </file>
@@ -440,16 +446,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C04845A8-D2B3-4AA5-B1E2-4210EB6AE0BD}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="39.5859375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.9375" customWidth="1"/>
-    <col min="4" max="4" width="36.5859375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.76171875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.87890625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.46875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.5859375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -460,10 +467,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A2">
         <v>0</v>
       </c>
@@ -474,11 +484,15 @@
         <f>500000000</f>
         <v>500000000</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2">
+        <f>230400000</f>
+        <v>230400000</v>
+      </c>
+      <c r="E2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.5">
       <c r="A3">
         <v>1</v>
       </c>
@@ -489,8 +503,28 @@
         <f>320000000</f>
         <v>320000000</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3">
+        <f t="shared" ref="D3:D4" si="0">230400000</f>
+        <v>230400000</v>
+      </c>
+      <c r="E3" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.5">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4">
+        <f>360000000</f>
+        <v>360000000</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>230400000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>